<commit_message>
update framework to support parallel execution across browsers
</commit_message>
<xml_diff>
--- a/UsersData/UsersDataForSignUp.xlsx
+++ b/UsersData/UsersDataForSignUp.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="13128" windowHeight="3792"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="RegisterUser" sheetId="1" r:id="rId1"/>
@@ -53,16 +53,16 @@
     <t>zip</t>
   </si>
   <si>
-    <t>Rohan</t>
+    <t>Rakesh</t>
   </si>
   <si>
     <t>Run</t>
   </si>
   <si>
-    <t>rohanrun111@test.com</t>
-  </si>
-  <si>
-    <t>Rohan@123</t>
+    <t>rakeshrun111@test.com</t>
+  </si>
+  <si>
+    <t>Rakesh@123</t>
   </si>
   <si>
     <t>Karve Nagar</t>
@@ -74,16 +74,16 @@
     <t>Pune</t>
   </si>
   <si>
-    <t>Sham</t>
+    <t>Mahesh</t>
   </si>
   <si>
     <t>Kontas</t>
   </si>
   <si>
-    <t>shamkontas22@test.com</t>
-  </si>
-  <si>
-    <t>Sham@123</t>
+    <t>maheshkontas22@test.com</t>
+  </si>
+  <si>
+    <t>Mahesh@123</t>
   </si>
   <si>
     <t>Baner</t>
@@ -1288,10 +1288,10 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" display="rohanrun111@test.com" tooltip="mailto:rohanrun111@test.com"/>
-    <hyperlink ref="C3" r:id="rId2" display="shamkontas22@test.com" tooltip="mailto:shamkontas22@test.com"/>
-    <hyperlink ref="D2" r:id="rId3" display="Rohan@123" tooltip="mailto:Rohan@123"/>
-    <hyperlink ref="D3" r:id="rId4" display="Sham@123" tooltip="mailto:Sham@123"/>
+    <hyperlink ref="C2" r:id="rId1" display="rakeshrun111@test.com" tooltip="mailto:rakeshrun111@test.com"/>
+    <hyperlink ref="C3" r:id="rId2" display="maheshkontas22@test.com" tooltip="mailto:maheshkontas22@test.com"/>
+    <hyperlink ref="D2" r:id="rId3" display="Rakesh@123" tooltip="mailto:Rakesh@123"/>
+    <hyperlink ref="D3" r:id="rId4" display="Mahesh@123" tooltip="mailto:Mahesh@123"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>